<commit_message>
chore(cascade): gbp_audit sheet → master template (header_row 3) + portfolio priority max 10→50
Closes FIX-J's two flagged out-of-scope gaps (manager cascade per the one-pass
additive-column/sheet memory): (1) templates/master-excel.xlsx gains the
gbp_audit sheet (7 headers, row 3 per schema) — template now carries all 19
schema sheets; FIX-J's KNOWN_SCHEMA_ONLY_SHEETS tripwire emptied by design.
(2) portfolio-config priority maximum 10→50: live portfolio legitimately
reached priority 12 (12 projects; mirrors the 8→12 maxItems precedent) —
shared/portfolio.json now validates clean (was 2 pre-existing errors).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/master-excel.xlsx
+++ b/templates/master-excel.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="redirect_404" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="completed_work" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="master_task" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gbp_audit" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -926,6 +927,57 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>audit_id</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>audit_date</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>gap_description</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>recommended_action</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>